<commit_message>
manual density for snowpro and densitycutter with mean
</commit_message>
<xml_diff>
--- a/code_automated_correlation/raw_data/20250321-densitycutter.xlsx
+++ b/code_automated_correlation/raw_data/20250321-densitycutter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\code_automated_correlation\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA6C691-2338-4163-BB97-F59FF0128D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C059796-3D8B-46F3-94EB-9283E019D01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FC14D368-F54E-477D-9C66-9A96069A1AC9}"/>
+    <workbookView xWindow="2520" yWindow="2810" windowWidth="14400" windowHeight="7270" xr2:uid="{FC14D368-F54E-477D-9C66-9A96069A1AC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>snowdepth</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Nan</t>
   </si>
   <si>
-    <t xml:space="preserve">mean </t>
-  </si>
-  <si>
     <t xml:space="preserve"> in kg/m^3</t>
   </si>
   <si>
@@ -69,6 +66,12 @@
   </si>
   <si>
     <t>density4</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>NaN</t>
   </si>
 </sst>
 </file>
@@ -466,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -475,7 +478,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
@@ -484,10 +487,10 @@
         <v>5</v>
       </c>
       <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
         <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -506,7 +509,7 @@
         <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -577,7 +580,7 @@
         <v>6</v>
       </c>
       <c r="I5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>